<commit_message>
Actualizar CPF-2 con tasas de fuga confirmadas (58.38 kg/Hr total)
</commit_message>
<xml_diff>
--- a/Emisiones-CPF1-CPF2-Organizado.xlsx
+++ b/Emisiones-CPF1-CPF2-Organizado.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="77">
   <si>
     <t xml:space="preserve">Registro de Emisiones Fugitivas — CPF-1</t>
   </si>
@@ -153,52 +153,64 @@
     <t xml:space="preserve">300-TK-0301</t>
   </si>
   <si>
-    <t xml:space="preserve">Manhole de 24" con escotilla cerrada pero empaque obstruido.</t>
+    <t xml:space="preserve">Manhole de 24" con escotilla cerrada pero empaque obstruido. Tasa medida: 540 g/Hr.</t>
   </si>
   <si>
     <t xml:space="preserve">300-TK-0201</t>
   </si>
   <si>
-    <t xml:space="preserve">Escotilla de 8" con empaque obstruido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manhole de 20" con escotilla cerrada pero empaque obstruido.</t>
+    <t xml:space="preserve">Escotilla de 8" con empaque obstruido. Tasa medida: 1.900 g/Hr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manhole de 20" con escotilla cerrada pero empaque obstruido. Tasa medida: 1.100 g/Hr.</t>
   </si>
   <si>
     <t xml:space="preserve">BRIDA</t>
   </si>
   <si>
-    <t xml:space="preserve">Brida / escotilla de 8" con empaque obstruido.</t>
+    <t xml:space="preserve">Brida / escotilla de 8" con empaque obstruido. Tasa medida: 750 g/Hr.</t>
   </si>
   <si>
     <t xml:space="preserve">300-TK-0101</t>
   </si>
   <si>
+    <t xml:space="preserve">Manhole de 20" con escotilla cerrada pero empaque obstruido. Tasa medida: 510 g/Hr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manhole de 24" con escotilla cerrada pero empaque obstruido. Tasa medida: 250 g/Hr.</t>
+  </si>
+  <si>
     <t xml:space="preserve">300-TK-0001</t>
   </si>
   <si>
+    <t xml:space="preserve">Manhole de 24" con escotilla cerrada pero empaque obstruido. Tasa medida: 300 g/Hr.</t>
+  </si>
+  <si>
     <t xml:space="preserve">300-TK-0401</t>
   </si>
   <si>
+    <t xml:space="preserve">Manhole de 20" con escotilla cerrada pero empaque obstruido. Tasa medida: 280 g/Hr.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALMACENAMIENTO</t>
   </si>
   <si>
     <t xml:space="preserve">300-TK-0103</t>
   </si>
   <si>
+    <t xml:space="preserve">Manhole de 24" con escotilla cerrada pero empaque obstruido. Tasa medida: 270 g/Hr.</t>
+  </si>
+  <si>
     <t xml:space="preserve">BRIDA INSTRUMENTACION</t>
   </si>
   <si>
     <t xml:space="preserve">EMPAQUE Y PERNOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Brida de instrumentación de 10": empaque obstruido y falta de pernos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manhole de 10": escotilla cerrada y sin empaque.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nota: el archivo fuente de CPF-2 no incluye tasa de fuga medida (g/Hr) en el texto ni de forma confiable en las fotos; columna omitida hasta confirmar los valores del medidor.</t>
+    <t xml:space="preserve">Brida de instrumentación de 10": empaque obstruido y falta de pernos. Tasa medida: 3.400 g/Hr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manhole de 10": escotilla cerrada y sin empaque. Tasa medida: 2.800 g/Hr.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumen — Emisiones Fugitivas CPF-1 y CPF-2</t>
@@ -211,6 +223,9 @@
   </si>
   <si>
     <t xml:space="preserve">Puntos de fuga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa total (g/Hr)</t>
   </si>
   <si>
     <t xml:space="preserve">CPF-1</t>
@@ -248,7 +263,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,14 +326,6 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF6E2C1F"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="9"/>
-      <color rgb="FF808080"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -408,7 +415,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -445,10 +452,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -457,7 +460,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1101,13 +1104,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>351360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1142640</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1123,7 +1126,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="952560"/>
+          <a:off x="7400880" y="952560"/>
           <a:ext cx="1142640" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1138,13 +1141,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>855720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1142640</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1160,7 +1163,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="1838160"/>
+          <a:off x="7400880" y="1838160"/>
           <a:ext cx="1142640" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1175,13 +1178,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1133280</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1197,7 +1200,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="2724120"/>
+          <a:off x="7400880" y="2724120"/>
           <a:ext cx="1133280" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1212,13 +1215,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1171080</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1234,7 +1237,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="3610080"/>
+          <a:off x="7400880" y="3610080"/>
           <a:ext cx="1171080" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1249,13 +1252,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>855720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1171080</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1271,7 +1274,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="4495680"/>
+          <a:off x="7400880" y="4495680"/>
           <a:ext cx="1171080" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1286,13 +1289,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1152000</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1308,7 +1311,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="5381640"/>
+          <a:off x="7400880" y="5381640"/>
           <a:ext cx="1152000" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1323,13 +1326,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1142640</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>827280</xdr:rowOff>
@@ -1345,7 +1348,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="6267600"/>
+          <a:off x="7400880" y="6267600"/>
           <a:ext cx="1142640" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1360,13 +1363,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1123560</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1382,7 +1385,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="7153200"/>
+          <a:off x="7400880" y="7153200"/>
           <a:ext cx="1123560" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1397,13 +1400,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1142640</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1419,7 +1422,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="8039160"/>
+          <a:off x="7400880" y="8039160"/>
           <a:ext cx="1142640" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1434,13 +1437,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>855720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1133280</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1456,7 +1459,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="8924760"/>
+          <a:off x="7400880" y="8924760"/>
           <a:ext cx="1133280" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1471,13 +1474,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>856080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>1142640</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>826920</xdr:rowOff>
@@ -1493,7 +1496,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6414120" y="9810720"/>
+          <a:off x="7400880" y="9810720"/>
           <a:ext cx="1142640" cy="856800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1527,17 +1530,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RegistroCPF2" displayName="RegistroCPF2" ref="A4:H15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A4:H15"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RegistroCPF2" displayName="RegistroCPF2" ref="A4:I15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A4:I15"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="N°"/>
     <tableColumn id="2" name="Área Específica"/>
     <tableColumn id="3" name="Equipo Sistema"/>
     <tableColumn id="4" name="Punto detectado"/>
     <tableColumn id="5" name="Elemento que fuga"/>
     <tableColumn id="6" name="Diametro (in)"/>
-    <tableColumn id="7" name="Evidencia"/>
-    <tableColumn id="8" name="Hallazgo"/>
+    <tableColumn id="7" name="Tasa fuga (g/Hr)"/>
+    <tableColumn id="8" name="Evidencia"/>
+    <tableColumn id="9" name="Hallazgo"/>
   </tableColumns>
 </table>
 </file>
@@ -2185,7 +2189,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2193,8 +2197,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2208,6 +2213,7 @@
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -2220,6 +2226,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
@@ -2241,9 +2248,12 @@
         <v>7</v>
       </c>
       <c r="G4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2266,8 +2276,11 @@
       <c r="F5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="5" t="s">
+      <c r="G5" s="4" t="n">
+        <v>540</v>
+      </c>
+      <c r="H5" s="4"/>
+      <c r="I5" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2290,8 +2303,11 @@
       <c r="F6" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="5" t="s">
+      <c r="G6" s="4" t="n">
+        <v>1900</v>
+      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="5" t="s">
         <v>45</v>
       </c>
     </row>
@@ -2314,8 +2330,11 @@
       <c r="F7" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="5" t="s">
+      <c r="G7" s="4" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2338,8 +2357,11 @@
       <c r="F8" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="5" t="s">
+      <c r="G8" s="4" t="n">
+        <v>750</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="5" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2362,9 +2384,12 @@
       <c r="F9" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="5" t="s">
-        <v>46</v>
+      <c r="G9" s="4" t="n">
+        <v>510</v>
+      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2386,9 +2411,12 @@
       <c r="F10" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="5" t="s">
-        <v>43</v>
+      <c r="G10" s="4" t="n">
+        <v>250</v>
+      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2399,7 +2427,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>16</v>
@@ -2410,9 +2438,12 @@
       <c r="F11" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="5" t="s">
-        <v>43</v>
+      <c r="G11" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H11" s="4"/>
+      <c r="I11" s="5" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2423,7 +2454,7 @@
         <v>23</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>16</v>
@@ -2434,9 +2465,12 @@
       <c r="F12" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G12" s="4"/>
-      <c r="H12" s="5" t="s">
-        <v>46</v>
+      <c r="G12" s="4" t="n">
+        <v>280</v>
+      </c>
+      <c r="H12" s="4"/>
+      <c r="I12" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2444,10 +2478,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>16</v>
@@ -2458,9 +2492,12 @@
       <c r="F13" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="G13" s="4"/>
-      <c r="H13" s="5" t="s">
-        <v>43</v>
+      <c r="G13" s="4" t="n">
+        <v>270</v>
+      </c>
+      <c r="H13" s="4"/>
+      <c r="I13" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2468,23 +2505,26 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="5" t="s">
-        <v>56</v>
+      <c r="G14" s="4" t="n">
+        <v>3400</v>
+      </c>
+      <c r="H14" s="4"/>
+      <c r="I14" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2492,10 +2532,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>16</v>
@@ -2506,20 +2546,18 @@
       <c r="F15" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
-        <v>58</v>
+      <c r="G15" s="4" t="n">
+        <v>2800</v>
+      </c>
+      <c r="H15" s="4"/>
+      <c r="I15" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2549,306 +2587,321 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
-        <v>60</v>
+      <c r="A3" s="8" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>62</v>
+      <c r="A4" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B5" s="11" t="n">
+      <c r="A5" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="10" t="n">
         <f aca="false">COUNTA(RegistroCPF1[N°])</f>
         <v>14</v>
       </c>
+      <c r="C5" s="10" t="n">
+        <f aca="false">SUM(RegistroCPF1[Tasa fuga (g/Hr)])</f>
+        <v>46278</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="11" t="n">
+      <c r="A6" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="10" t="n">
         <f aca="false">COUNTA(RegistroCPF2[N°])</f>
         <v>11</v>
       </c>
+      <c r="C6" s="10" t="n">
+        <f aca="false">SUM(RegistroCPF2[Tasa fuga (g/Hr)])</f>
+        <v>12100</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="12" t="n">
+      <c r="A7" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="11" t="n">
         <f aca="false">B5+B6</f>
         <v>25</v>
       </c>
+      <c r="C7" s="11" t="n">
+        <f aca="false">C5+C6</f>
+        <v>58378</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>66</v>
+      <c r="A9" s="8" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>68</v>
+      <c r="A10" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="13" t="n">
+      <c r="B11" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Área Específica],A11)</f>
         <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Área Específica],A12)</f>
         <v>7</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="13" t="n">
+      <c r="B13" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Área Específica],A13)</f>
         <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B14" s="12" t="n">
+      <c r="A14" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="11" t="n">
         <f aca="false">SUM(B11:B13)</f>
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>69</v>
+      <c r="A16" s="8" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>68</v>
+      <c r="A17" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A18)</f>
         <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A19)</f>
         <v>2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="13" t="n">
+      <c r="B20" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A20)</f>
         <v>2</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="13" t="n">
+      <c r="B21" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A21)</f>
         <v>4</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="13" t="n">
+      <c r="B22" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A22)</f>
         <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A23)</f>
         <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A24)</f>
         <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF1[Equipo Sistema],A25)</f>
         <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B26" s="12" t="n">
+      <c r="A26" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="11" t="n">
         <f aca="false">SUM(B18:B25)</f>
         <v>14</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9" t="s">
-        <v>70</v>
+      <c r="A28" s="8" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>68</v>
+      <c r="A29" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B30" s="13" t="n">
+      <c r="A30" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Área Específica],A30)</f>
         <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="13" t="n">
+      <c r="B31" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Área Específica],A31)</f>
         <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B32" s="12" t="n">
+      <c r="A32" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="11" t="n">
         <f aca="false">SUM(B30:B31)</f>
         <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9" t="s">
-        <v>71</v>
+      <c r="A34" s="8" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>68</v>
+      <c r="A35" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="B36" s="13" t="n">
+      <c r="A36" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A36)</f>
         <v>1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
+      <c r="A37" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B37" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A37)</f>
         <v>2</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B38" s="13" t="n">
+      <c r="A38" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A38)</f>
         <v>3</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B39" s="13" t="n">
+      <c r="B39" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A39)</f>
         <v>3</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
+      <c r="A40" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="B40" s="13" t="n">
+      <c r="B40" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A40)</f>
         <v>1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B41" s="13" t="n">
+      <c r="A41" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="12" t="n">
         <f aca="false">COUNTIF(RegistroCPF2[Equipo Sistema],A41)</f>
         <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="B42" s="12" t="n">
+      <c r="A42" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B42" s="11" t="n">
         <f aca="false">SUM(B36:B41)</f>
         <v>11</v>
       </c>

</xml_diff>